<commit_message>
+= get_all_product_image api + header optimisations
</commit_message>
<xml_diff>
--- a/backend tests.xlsx
+++ b/backend tests.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="328">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -58,7 +58,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="1"/>
@@ -68,7 +68,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="238"/>
@@ -78,7 +78,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="1"/>
@@ -226,7 +226,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="1"/>
@@ -236,7 +236,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="238"/>
@@ -246,7 +246,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="1"/>
@@ -802,6 +802,267 @@
   </si>
   <si>
     <t xml:space="preserve">T-54,T-55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/update_user_state_admin works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/update_user_state_admin/ with the body {  "admin_id": "&lt;b64 encoded admin user id&gt;",  "admin_session_token": "&lt;b64 encoded admin session token&gt;"   "target_user_id":"&lt;b64 enc. id of targed user&gt;",  "new_user_state":"&lt;b64 enc. desired user state&gt;",  "reason":"&lt;b64 enc. ban reason ! only if the new user state is banned !&gt;"}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-58,T-59,T-60,T-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/update_user_state_admin works (wrong permissions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/update_user_state_admin/ with the body {  "admin_id": "&lt;b64 encoded NON ADMIN id&gt;",  "admin_session_token": "&lt;b64 encoded NON ADMIN session token&gt;"   "target_user_id":"&lt;b64 enc. id of targed user&gt;",  "new_user_state":"&lt;b64 enc. desired user state&gt;",  "reason":"&lt;b64 enc. ban reason ! only if the new user state is banned !&gt;"}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response: 403 (FORBIDDEN), body: „{     "status": "permission_denied",     "statuscode": "403" }"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-57,T-59,T-60,T-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/update_user_state_admin works (wrong token)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/update_user_state_admin/ with the body {  "admin_id": "&lt;b64 encoded admin id&gt;",  "admin_session_token": "&lt;b64 encoded WRONG admin session token&gt;"   "target_user_id":"&lt;b64 enc. id of targed user&gt;",  "new_user_state":"&lt;b64 enc. desired user state&gt;",  "reason":"&lt;b64 enc. ban reason ! only if the new user state is banned !&gt;"}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response: 401 (UNATHORIZED), body: „{     "status": "incorrect_credentials",     "statuscode": "401" }"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-57,T-58,T-60,T-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/update_user_state_admin works (no jwt provided)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/update_user_state_admin/ with the body {  "admin_id": "&lt;b64 encoded admin id&gt;",  "admin_session_token": "&lt;b64 encoded admin session token&gt;"   "target_user_id":"&lt;b64 enc. id of targed user&gt;",  "new_user_state":"&lt;b64 enc. desired user state&gt;",  "reason":"&lt;b64 enc. ban reason ! only if the new user state is banned !&gt;"}, without an auth header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response: 401 (UNATHORIZED), body: „{"status":"missing_auth_header","statuscode":"401"}"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-57,T-58,T-59,T-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/update_user_state_admin works (missing fields)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/update_user_state_admin/ with the body {  "admin_id": "&lt;b64 encoded admin id&gt;",  "admin_session_token": "&lt;b64 encoded admin session token&gt;"   "target_user_id":"&lt;b64 enc. id of targed user&gt;",  "reason":"&lt;b64 enc. ban reason ! only if the new user state is banned !&gt;"}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-57,T-58,T-59,T-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-62</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_product works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/create_product/ with the body {  "admin_id": "&lt;b64 encoded admin user {   "user_id": "&lt;base64 enc. id of admin&gt;",    "session_token": "&lt;base64 enc. session token of admin&gt;",    "name_de":"&lt;b64 enc. string&gt;",    "description_en":"&lt;b64 enc. string&gt;",    "price_huf":"&lt;b64 enc. int&gt;",   "times_ordered":"&lt;b64 enc. int&gt;",    "stock":"&lt;b64 enc. int&gt;",   "sale_percentage":"&lt;b64 enc. int&gt;",    "description_preview_en":"&lt;b64 enc. string&gt;",     "name_hu":"&lt;b64 enc. string&gt;",     "name_en":"&lt;b64 enc. string&gt;",    "description_hu":"&lt;b64 enc. string&gt;",    "description_de":"&lt;b64 enc. string&gt;",     "description_preview_hu":"&lt;b64 enc. string&gt;",    "description_preview_de":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",  "manufacturer":"&lt;b64 enc. string&gt;",   "brand":"&lt;b64 enc. string&gt;",  "rating":"&lt;b64 enc. int&gt;",  "sku":"&lt;b64 enc. string&gt;",   "active_ingredients":"&lt;b64 enc. string&gt;",   "packaging_en":"&lt;b64 enc. string&gt;",   "packaging_hu":"&lt;b64 enc. string&gt;",  "packaging_de":"&lt;b64 enc. string&gt;",  "thumbnail_url":"&lt;b64 enc. string&gt;", "featured":"&lt;b64 enc. Int&gt;"  }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-64, T-65, T-65, T-66, T-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_product works (not admin user)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/create_product/ with the body {  "admin_id": "&lt;b64 encoded admin user {   "user_id": "&lt;base64 encNOT . id of admin&gt;",    "session_token": "&lt;base64 enc. session token of admin&gt;",    "name_de":"&lt;b64 enc. Strina NOT g&gt;",  user   "description_en":"&lt;b64 enc. string&gt;",    "price_huf":"&lt;b64 enc. int&gt;",   "times_ordered":"&lt;b64 enc. int&gt;",    "stock":"&lt;b64 enc. int&gt;",   "sale_percentage":"&lt;b64 enc. int&gt;",    "description_preview_en":"&lt;b64 enc. string&gt;",     "name_hu":"&lt;b64 enc. string&gt;",     "name_en":"&lt;b64 enc. string&gt;",    "description_hu":"&lt;b64 enc. string&gt;",    "description_de":"&lt;b64 enc. string&gt;",     "description_preview_hu":"&lt;b64 enc. string&gt;",    "description_preview_de":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",  "manufacturer":"&lt;b64 enc. string&gt;",   "brand":"&lt;b64 enc. string&gt;",  "rating":"&lt;b64 enc. int&gt;",  "sku":"&lt;b64 enc. string&gt;",   "active_ingredients":"&lt;b64 enc. string&gt;",   "packaging_en":"&lt;b64 enc. string&gt;",   "packaging_hu":"&lt;b64 enc. string&gt;",  "packaging_de":"&lt;b64 enc. string&gt;",  "thumbnail_url":"&lt;b64 enc. string&gt;", "featured":"&lt;b64 enc. Int&gt;"  }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-62, T-64, T-65, T-66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_product works (wrong token)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/create_product/ with the body {  "admin_id": "&lt;b64 encoded admin user {   "user_id": "&lt;base64 enc. id of admin&gt;",    "session_token": "&lt;base64 enc. INCORRECT session token of admin&gt;",    "name_de":"&lt;b64 enc. string&gt;",    "description_en":"&lt;b64 enc. string&gt;",    "price_huf":"&lt;b64 enc. int&gt;",   "times_ordered":"&lt;b64 enc. int&gt;",    "stock":"&lt;b64 enc. int&gt;",   "sale_percentage":"&lt;b64 enc. int&gt;",    "description_preview_en":"&lt;b64 enc. string&gt;",     "name_hu":"&lt;b64 enc. string&gt;",     "name_en":"&lt;b64 enc. string&gt;",    "description_hu":"&lt;b64 enc. string&gt;",    "description_de":"&lt;b64 enc. string&gt;",     "description_preview_hu":"&lt;b64 enc. string&gt;",    "description_preview_de":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",  "manufacturer":"&lt;b64 enc. string&gt;",   "brand":"&lt;b64 enc. string&gt;",  "rating":"&lt;b64 enc. int&gt;",  "sku":"&lt;b64 enc. string&gt;",   "active_ingredients":"&lt;b64 enc. string&gt;",   "packaging_en":"&lt;b64 enc. string&gt;",   "packaging_hu":"&lt;b64 enc. string&gt;",  "packaging_de":"&lt;b64 enc. string&gt;",  "thumbnail_url":"&lt;b64 enc. string&gt;", "featured":"&lt;b64 enc. Int&gt;"  }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-62, T-63, T-65, T-66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_product works (no jwt provided)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/create_product/ with the body {  "admin_id": "&lt;b64 encoded admin user {   "user_id": "&lt;base64 enc. id of admin&gt;",    "session_token": "&lt;base64 enc. session token of admin&gt;",    "name_de":"&lt;b64 enc. string&gt;",    "description_en":"&lt;b64 enc. string&gt;",    "price_huf":"&lt;b64 enc. int&gt;",   "times_ordered":"&lt;b64 enc. int&gt;",    "stock":"&lt;b64 enc. int&gt;",   "sale_percentage":"&lt;b64 enc. int&gt;",    "description_preview_en":"&lt;b64 enc. string&gt;",     "name_hu":"&lt;b64 enc. string&gt;",     "name_en":"&lt;b64 enc. string&gt;",    "description_hu":"&lt;b64 enc. string&gt;",    "description_de":"&lt;b64 enc. string&gt;",     "description_preview_hu":"&lt;b64 enc. string&gt;",    "description_preview_de":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",  "manufacturer":"&lt;b64 enc. string&gt;",   "brand":"&lt;b64 enc. string&gt;",  "rating":"&lt;b64 enc. int&gt;",  "sku":"&lt;b64 enc. string&gt;",   "active_ingredients":"&lt;b64 enc. string&gt;",   "packaging_en":"&lt;b64 enc. string&gt;",   "packaging_hu":"&lt;b64 enc. string&gt;",  "packaging_de":"&lt;b64 enc. string&gt;",  "thumbnail_url":"&lt;b64 enc. string&gt;", "featured":"&lt;b64 enc. Int&gt;"  }, and no header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-62, T-63, T-64, T-66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_product works (missing fields)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to  http://localhost:90/api/create_product/ with the body {  "admin_id": "&lt;b64 encoded admin user {   "user_id": "&lt;base64 enc. id of admin&gt;",    "session_token": "&lt;base64 enc. session token of admin&gt;",    "name_de":"&lt;b64 enc. string&gt;",    "description_en":"&lt;b64 enc. string&gt;",    "price_huf":"&lt;b64 enc. int&gt;",   "times_ordered":"&lt;b64 enc. int&gt;",    "stock":"&lt;b64 enc. int&gt;",   "sale_percentage":"&lt;b64 enc. int&gt;",    "description_preview_en":"&lt;b64 enc. string&gt;",     "name_hu":"&lt;b64 enc. string&gt;",     "name_en":"&lt;b64 enc. string&gt;",    "description_hu":"&lt;b64 enc. string&gt;",    "description_de":"&lt;b64 enc. string&gt;",     "description_preview_hu":"&lt;b64 enc. string&gt;",    "description_preview_de":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",  "manufacturer":"&lt;b64 enc. string&gt;",   "brand":"&lt;b64 enc. string&gt;",  "rating":"&lt;b64 enc. int&gt;",  "sku":"&lt;b64 enc. string&gt;",   "active_ingredients":"&lt;b64 enc. string&gt;",   "packaging_en":"&lt;b64 enc. String&gt;"  }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-62, T-63, T-64, T-65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_order works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_order with the body {   "order": {     "user_id": "&lt;b64 enc. id of user&gt;",     "session_token": "&lt;b64 enc.  Session token of user&gt;",     "email": "&lt;b64 enc. email of user&gt;",     "billing_name": "&lt;64 enc. string&gt;",     "shipping_name": "&lt;64 enc. string&gt;",     "shipping_company": "&lt;64 enc. string&gt;",     "price": "&lt;64 enc. int&gt;",     "city": "&lt;64 enc. string&gt;",     "guest": "&lt;64 enc. int (0,1)&gt;",     "zipcode": "&lt;64 enc. int&gt;",     "address": "&lt;64 enc. string&gt;",     "apartment_number": "&lt;64 enc. int&gt;",     "note": "&lt;64 enc. string&gt;",     "house_number": "&lt;64 enc. int&gt;",     "phone_number": "&lt;64 enc. string&gt;"   },   "items": [     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"         },     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"           }   ] }   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response: 200 (SUCCESS), body: „{"status":"success","statuscode":"200","tracking_token":"&lt;the order’s tracking token&gt;"}"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-68,T-69,T-70,T-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_order works (banned user)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_order with the body {   "order": {     "user_id": "&lt;b64 enc. id of a BANNED user&gt;",     "session_token": "&lt;b64 enc.  Session token of user&gt;",     "email": "&lt;b64 enc. email of user&gt;",     "billing_name": "&lt;64 enc. string&gt;",     "shipping_name": "&lt;64 enc. string&gt;",     "shipping_company": "&lt;64 enc. string&gt;",     "price": "&lt;64 enc. int&gt;",     "city": "&lt;64 enc. string&gt;",     "guest": "&lt;64 enc. int (0,1)&gt;",     "zipcode": "&lt;64 enc. int&gt;",     "address": "&lt;64 enc. string&gt;",     "apartment_number": "&lt;64 enc. int&gt;",     "note": "&lt;64 enc. string&gt;",     "house_number": "&lt;64 enc. int&gt;",     "phone_number": "&lt;64 enc. string&gt;"   },   "items": [     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"         },     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"           }   ] }   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response: 403 (FORBIDDEN), body: „{"status":"permission_denied","statuscode":"403"}"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-67,T-69,T-70,T-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_order works (wrong token)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_order with the body {   "order": {     "user_id": "&lt;b64 enc. id of user&gt;",     "session_token": "&lt;b64 enc. INCORRECT Session token of user&gt;",     "email": "&lt;b64 enc. email of user&gt;",     "billing_name": "&lt;64 enc. string&gt;",     "shipping_name": "&lt;64 enc. string&gt;",     "shipping_company": "&lt;64 enc. string&gt;",     "price": "&lt;64 enc. int&gt;",     "city": "&lt;64 enc. string&gt;",     "guest": "&lt;64 enc. int (0,1)&gt;",     "zipcode": "&lt;64 enc. int&gt;",     "address": "&lt;64 enc. string&gt;",     "apartment_number": "&lt;64 enc. int&gt;",     "note": "&lt;64 enc. string&gt;",     "house_number": "&lt;64 enc. int&gt;",     "phone_number": "&lt;64 enc. string&gt;"   },   "items": [     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"         },     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"           }   ] }   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response: 401 (UNATHORIZED), body: „{"status":"incorrect_credentials","statuscode":"401"}"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-67,T-68,T-70,T-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_order works (no jwt provided)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_order with the body {   "order": {     "user_id": "&lt;b64 enc. id of user&gt;",     "session_token": "&lt;b64 enc.  Session token of user&gt;",     "email": "&lt;b64 enc. email of user&gt;",     "billing_name": "&lt;64 enc. string&gt;",     "shipping_name": "&lt;64 enc. string&gt;",     "shipping_company": "&lt;64 enc. string&gt;",     "price": "&lt;64 enc. int&gt;",     "city": "&lt;64 enc. string&gt;",     "guest": "&lt;64 enc. int (0,1)&gt;",     "zipcode": "&lt;64 enc. int&gt;",     "address": "&lt;64 enc. string&gt;",     "apartment_number": "&lt;64 enc. int&gt;",     "note": "&lt;64 enc. string&gt;",     "house_number": "&lt;64 enc. int&gt;",     "phone_number": "&lt;64 enc. string&gt;"   },   "items": [     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"         },     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. Int&gt;"           }   ] }, and no header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-67,T-68,T-69,T-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_order works (missing fields)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_order with the body {   "order": {     "user_id": "&lt;b64 enc. id of user&gt;",     "session_token": "&lt;b64 enc.  Session token of user&gt;",     "email": "&lt;b64 enc. email of user&gt;",     "billing_name": "&lt;64 enc. string&gt;",     "shipping_name": "&lt;64 enc. string&gt;",     "shipping_company": "&lt;64 enc. string&gt;",     "price": "&lt;64 enc. int&gt;",     "city": "&lt;64 enc. String&gt;",    "address": "&lt;64 enc. string&gt;",     "apartment_number": "&lt;64 enc. int&gt;",     "note": "&lt;64 enc. string&gt;",     "house_number": "&lt;64 enc. int&gt;",     "phone_number": "&lt;64 enc. string&gt;"   },   "items": [     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"         },     {       "product_id": "&lt;64 enc. int&gt;",       "quantity": "&lt;64 enc. int&gt;"           }   ] }   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-67,T-68,T-69,T-70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_post works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_post with the body: {   "user_id": "&lt;b64 enc. id of admin&gt;",   "session_token": ""&lt;b64 enc. session token of admin&gt;",   "title":""&lt;b64 enc. string&gt;",    "content":"&lt;b64 enc. string&gt;",    "image_url":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",   "slug":"&lt;b64 enc. string&gt;",   "except":"&lt;b64 enc. string&gt;",    "status":"&lt;b64 enc. string (hidden, draft, published, archived)&gt;",   "views":"&lt;b64 enc. int&gt;",    "likes":"&lt;b64 enc. int&gt;",   "comment_count":"&lt;b64 enc. int&gt;",    "is_featured":"&lt;b64 enc. int (0,1)&gt;",    "tags":"&lt;b64 enc. string&gt;" }   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response: 200 (SUCCESS), body: „{"status":"success","statuscode":"200"}"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-73,T-74,T-75,T-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-73</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_post works (missing admin priviliges)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_post with the body: {   "user_id": "&lt;b64 enc. id of NON-ADMIN user&gt;",   "session_token": ""&lt;b64 enc. session token of NON-ADMIN user&gt;",   "title":""&lt;b64 enc. string&gt;",    "content":"&lt;b64 enc. string&gt;",    "image_url":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",   "slug":"&lt;b64 enc. string&gt;",   "except":"&lt;b64 enc. string&gt;",    "status":"&lt;b64 enc. string (hidden, draft, published, archived)&gt;",   "views":"&lt;b64 enc. int&gt;",    "likes":"&lt;b64 enc. int&gt;",   "comment_count":"&lt;b64 enc. int&gt;",    "is_featured":"&lt;b64 enc. int (0,1)&gt;",    "tags":"&lt;b64 enc. string&gt;" }   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-72,T-74,T-75,T-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_post works (wrong token)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_post with the body: {   "user_id": "&lt;b64 enc. id of admin&gt;",   "session_token": ""&lt;b64 enc. INCORRECT session token of admin&gt;",   "title":""&lt;b64 enc. string&gt;",    "content":"&lt;b64 enc. string&gt;",    "image_url":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",   "slug":"&lt;b64 enc. string&gt;",   "except":"&lt;b64 enc. string&gt;",    "status":"&lt;b64 enc. string (hidden, draft, published, archived)&gt;",   "views":"&lt;b64 enc. int&gt;",    "likes":"&lt;b64 enc. int&gt;",   "comment_count":"&lt;b64 enc. int&gt;",    "is_featured":"&lt;b64 enc. int (0,1)&gt;",    "tags":"&lt;b64 enc. string&gt;" }   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-73,T-72,T-75,T-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_post works (no jwt provided)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_post with the body: {   "user_id": "&lt;b64 enc. id of admin&gt;",   "session_token": ""&lt;b64 enc. session token of admin&gt;",   "title":""&lt;b64 enc. string&gt;",    "content":"&lt;b64 enc. string&gt;",    "image_url":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",   "slug":"&lt;b64 enc. string&gt;",   "except":"&lt;b64 enc. string&gt;",    "status":"&lt;b64 enc. string (hidden, draft, published, archived)&gt;",   "views":"&lt;b64 enc. int&gt;",    "likes":"&lt;b64 enc. int&gt;",   "comment_count":"&lt;b64 enc. int&gt;",    "is_featured":"&lt;b64 enc. int (0,1)&gt;",    "tags":"&lt;b64 enc. String&gt;" }, and no auth header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-73,T-74,T-72,T-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test if api/create_post works (missing fields)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open postman 2. Send a request to https://www.roysshack.hu/create_post with the body: {   "user_id": "&lt;b64 enc. id of admin&gt;",   "session_token": ""&lt;b64 enc. session token of admin&gt;",   "title":""&lt;b64 enc. string&gt;",    "content":"&lt;b64 enc. string&gt;",    "image_url":"&lt;b64 enc. string&gt;",   "category_id":"&lt;b64 enc. int&gt;",   "slug":"&lt;b64 enc. string&gt;",   "except":"&lt;b64 enc. string&gt;",    "status":"&lt;b64 enc. string (hidden, draft, published, archived)&gt;",   "views":"&lt;b64 enc. int&gt;",    "likes":"&lt;b64 enc. int&gt;",   "comment_count":"&lt;b64 enc. Int&gt;" }   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-73,T-74,T-75,T-72</t>
   </si>
 </sst>
 </file>
@@ -813,7 +1074,7 @@
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -841,31 +1102,24 @@
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="DejaVu Sans"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF81D41A"/>
-      <name val="DejaVu Sans"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -884,7 +1138,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor rgb="FF81D41A"/>
+        <bgColor rgb="FF339966"/>
       </patternFill>
     </fill>
     <fill>
@@ -946,7 +1200,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -991,15 +1245,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1056,7 +1306,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF81D41A"/>
+      <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFC000"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFC55A11"/>
@@ -1252,17 +1502,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V63"/>
+  <dimension ref="A1:V87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="46.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="77.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="57.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="33.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="21.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15.07"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.68"/>
   </cols>
@@ -2311,8 +2561,12 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="97.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
+      <c r="A37" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>150</v>
+      </c>
       <c r="C37" s="1" t="s">
         <v>25</v>
       </c>
@@ -3006,7 +3260,7 @@
       <c r="C61" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="D61" s="13" t="s">
+      <c r="D61" s="1" t="s">
         <v>228</v>
       </c>
       <c r="E61" s="1" t="s">
@@ -3081,6 +3335,586 @@
       </c>
       <c r="I63" s="12" t="n">
         <v>46079</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C65" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="G65" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="I65" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C66" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="I66" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C67" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="I67" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="I68" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C69" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="G69" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="I69" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C71" s="10" t="s">
+        <v>265</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="G71" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="I71" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C72" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G72" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I72" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C73" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G73" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I73" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="C74" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G74" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="I74" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C75" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="G75" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="I75" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="C77" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I77" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C78" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G78" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="I78" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="n">
+        <v>69</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="G79" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="I79" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C80" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G80" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="I80" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C81" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="G81" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="I81" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C83" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="G83" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="I83" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="C84" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="G84" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="I84" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="n">
+        <v>74</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="C85" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="G85" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="I85" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="C86" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G86" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H86" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="I86" s="12" t="n">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="n">
+        <v>76</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="C87" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="G87" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H87" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="I87" s="12" t="n">
+        <v>46104</v>
       </c>
     </row>
   </sheetData>
@@ -3089,6 +3923,16 @@
     <hyperlink ref="D51" r:id="rId2" display="1. Open postman 2. Send a request to  http://localhost:90/api/get_all_product_categories/ with the body  „ {    &quot;id&quot;: &quot;&lt;b64encoded id”, &quot;passwo"/>
     <hyperlink ref="D52" r:id="rId3" display="1. Open postman 2. Send a request to  http://localhost:90/api/get_all_product_categories/ without a body or an s_featured"/>
     <hyperlink ref="D53" r:id="rId4" display="1. Open postman 2. Send a request to  http://localhost:90/api/get_all_product_categories/ with the body  „ {    &quot;id&quot;: &quot;&lt;b64encoded i” "/>
+    <hyperlink ref="D71" r:id="rId5" display="http://localhost:90/api/create_product/"/>
+    <hyperlink ref="D72" r:id="rId6" display="http://localhost:90/api/create_product/"/>
+    <hyperlink ref="D73" r:id="rId7" display="http://localhost:90/api/create_product/"/>
+    <hyperlink ref="D74" r:id="rId8" display="http://localhost:90/api/create_product/"/>
+    <hyperlink ref="D75" r:id="rId9" display="http://localhost:90/api/create_product/"/>
+    <hyperlink ref="D83" r:id="rId10" display="https://www.roysshack.hu/create_post"/>
+    <hyperlink ref="D84" r:id="rId11" display="https://www.roysshack.hu/create_post"/>
+    <hyperlink ref="D85" r:id="rId12" display="https://www.roysshack.hu/create_post"/>
+    <hyperlink ref="D86" r:id="rId13" display="https://www.roysshack.hu/create_post"/>
+    <hyperlink ref="D87" r:id="rId14" display="https://www.roysshack.hu/create_post"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
cache fix + egyeb bug javitas
</commit_message>
<xml_diff>
--- a/backend tests.xlsx
+++ b/backend tests.xlsx
@@ -1473,7 +1473,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1524,6 +1524,10 @@
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -4229,15 +4233,15 @@
       </c>
     </row>
     <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A101" s="0"/>
-      <c r="B101" s="0"/>
-      <c r="C101" s="0"/>
-      <c r="D101" s="0"/>
-      <c r="E101" s="0"/>
-      <c r="F101" s="0"/>
-      <c r="G101" s="0"/>
-      <c r="H101" s="0"/>
-      <c r="I101" s="0"/>
+      <c r="A101" s="13"/>
+      <c r="B101" s="13"/>
+      <c r="C101" s="13"/>
+      <c r="D101" s="13"/>
+      <c r="E101" s="13"/>
+      <c r="F101" s="13"/>
+      <c r="G101" s="13"/>
+      <c r="H101" s="13"/>
+      <c r="I101" s="13"/>
     </row>
     <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
@@ -4264,7 +4268,7 @@
       <c r="H102" s="12" t="n">
         <v>46105</v>
       </c>
-      <c r="I102" s="0"/>
+      <c r="I102" s="13"/>
     </row>
     <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
@@ -4291,7 +4295,7 @@
       <c r="H103" s="12" t="n">
         <v>46105</v>
       </c>
-      <c r="I103" s="0"/>
+      <c r="I103" s="13"/>
     </row>
     <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
@@ -4318,7 +4322,7 @@
       <c r="H104" s="12" t="n">
         <v>46105</v>
       </c>
-      <c r="I104" s="0"/>
+      <c r="I104" s="13"/>
     </row>
     <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
@@ -4374,7 +4378,7 @@
     </row>
     <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B107" s="10"/>
-      <c r="F107" s="0"/>
+      <c r="F107" s="13"/>
       <c r="H107" s="12"/>
     </row>
     <row r="108" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4508,14 +4512,14 @@
       </c>
     </row>
     <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="0"/>
-      <c r="B113" s="0"/>
-      <c r="C113" s="0"/>
-      <c r="D113" s="0"/>
-      <c r="E113" s="0"/>
-      <c r="F113" s="0"/>
-      <c r="G113" s="0"/>
-      <c r="H113" s="0"/>
+      <c r="A113" s="13"/>
+      <c r="B113" s="13"/>
+      <c r="C113" s="13"/>
+      <c r="D113" s="13"/>
+      <c r="E113" s="13"/>
+      <c r="F113" s="13"/>
+      <c r="G113" s="13"/>
+      <c r="H113" s="13"/>
     </row>
     <row r="114" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="s">
@@ -4587,11 +4591,11 @@
     <hyperlink ref="C85" r:id="rId12" display="1. Open postman 2. Send a request to https://www.roysshack.hu/create_post with the body: {   &quot;user_id&quot;: &quot;&lt;b64 enc. id of admin&gt;&quot;,   &quot;session_token&quot;: &quot;&quot;&lt;b64 enc. INCORRECT session token of admin&gt;&quot;,   &quot;title&quot;:&quot;&quot;&lt;b64 enc. string&gt;&quot;,    &quot;content&quot;:&quot;&lt;b64 enc. string&gt;&quot;,    &quot;image_url&quot;:&quot;&lt;b64 enc. string&gt;&quot;,   &quot;category_id&quot;:&quot;&lt;b64 enc. int&gt;&quot;,   &quot;slug&quot;:&quot;&lt;b64 enc. string&gt;&quot;,   &quot;except&quot;:&quot;&lt;b64 enc. string&gt;&quot;,    &quot;status&quot;:&quot;&lt;b64 enc. string (hidden, draft, published, archived)&gt;&quot;,   &quot;views&quot;:&quot;&lt;b64 enc. int&gt;&quot;,    &quot;likes&quot;:&quot;&lt;b64 enc. int&gt;&quot;,   &quot;comment_count&quot;:&quot;&lt;b64 enc. int&gt;&quot;,    &quot;is_featured&quot;:&quot;&lt;b64 enc. int (0,1)&gt;&quot;,    &quot;tags&quot;:&quot;&lt;b64 enc. string&gt;&quot; }   "/>
     <hyperlink ref="C86" r:id="rId13" display="1. Open postman 2. Send a request to https://www.roysshack.hu/create_post with the body: {   &quot;user_id&quot;: &quot;&lt;b64 enc. id of admin&gt;&quot;,   &quot;session_token&quot;: &quot;&quot;&lt;b64 enc. session token of admin&gt;&quot;,   &quot;title&quot;:&quot;&quot;&lt;b64 enc. string&gt;&quot;,    &quot;content&quot;:&quot;&lt;b64 enc. string&gt;&quot;,    &quot;image_url&quot;:&quot;&lt;b64 enc. string&gt;&quot;,   &quot;category_id&quot;:&quot;&lt;b64 enc. int&gt;&quot;,   &quot;slug&quot;:&quot;&lt;b64 enc. string&gt;&quot;,   &quot;except&quot;:&quot;&lt;b64 enc. string&gt;&quot;,    &quot;status&quot;:&quot;&lt;b64 enc. string (hidden, draft, published, archived)&gt;&quot;,   &quot;views&quot;:&quot;&lt;b64 enc. int&gt;&quot;,    &quot;likes&quot;:&quot;&lt;b64 enc. int&gt;&quot;,   &quot;comment_count&quot;:&quot;&lt;b64 enc. int&gt;&quot;,    &quot;is_featured&quot;:&quot;&lt;b64 enc. int (0,1)&gt;&quot;,    &quot;tags&quot;:&quot;&lt;b64 enc. String&gt;&quot; }, and no auth header"/>
     <hyperlink ref="C87" r:id="rId14" display="1. Open postman 2. Send a request to https://www.roysshack.hu/create_post with the body: {   &quot;user_id&quot;: &quot;&lt;b64 enc. id of admin&gt;&quot;,   &quot;session_token&quot;: &quot;&quot;&lt;b64 enc. session token of admin&gt;&quot;,   &quot;title&quot;:&quot;&quot;&lt;b64 enc. string&gt;&quot;,    &quot;content&quot;:&quot;&lt;b64 enc. string&gt;&quot;,    &quot;image_url&quot;:&quot;&lt;b64 enc. string&gt;&quot;,   &quot;category_id&quot;:&quot;&lt;b64 enc. int&gt;&quot;,   &quot;slug&quot;:&quot;&lt;b64 enc. string&gt;&quot;,   &quot;except&quot;:&quot;&lt;b64 enc. string&gt;&quot;,    &quot;status&quot;:&quot;&lt;b64 enc. string (hidden, draft, published, archived)&gt;&quot;,   &quot;views&quot;:&quot;&lt;b64 enc. int&gt;&quot;,    &quot;likes&quot;:&quot;&lt;b64 enc. int&gt;&quot;,   &quot;comment_count&quot;:&quot;&lt;b64 enc. Int&gt;&quot; }   "/>
-    <hyperlink ref="C102" r:id="rId15" display="https://www.roysshack.hu/update_stock_admin"/>
-    <hyperlink ref="C103" r:id="rId16" display="https://www.roysshack.hu/update_stock_admin"/>
-    <hyperlink ref="C104" r:id="rId17" display="https://www.roysshack.hu/update_stock_admin"/>
-    <hyperlink ref="C105" r:id="rId18" display="https://www.roysshack.hu/update_stock_admin"/>
-    <hyperlink ref="C106" r:id="rId19" display="https://www.roysshack.hu/update_stock_admin"/>
+    <hyperlink ref="C102" r:id="rId15" display="1. Open postman 2. Send a request to https://www.roysshack.hu/update_stock_admin with the body {  &quot;user_id&quot;:&quot;&lt;b64 enc. id of user&gt;&quot;, &quot;session_token&quot;:&quot;&lt;b64 enc. session token of user&gt;&quot;, &quot;post_id&quot;:&quot;&lt;b64 enc. id of post&gt;&quot; }"/>
+    <hyperlink ref="C103" r:id="rId16" display="1. Open postman 2. Send a request to https://www.roysshack.hu/update_stock_admin with the body {  &quot;user_id&quot;:&quot;&lt;b64 enc. id of user&gt;&quot;, &quot;session_token&quot;:&quot;&lt;b64 enc. session token of user&gt;&quot;, &quot;post_id&quot;:&quot;&lt;b64 enc. id of post&gt;&quot; }"/>
+    <hyperlink ref="C104" r:id="rId17" display="1. Open postman 2. Send a request to https://www.roysshack.hu/update_stock_admin with the body {  &quot;user_id&quot;:&quot;&lt;b64 enc. id of user&gt;&quot;, &quot;session_token&quot;:&quot;&lt;b64 enc. INCORRECT session token of user&gt;&quot;, &quot;post_id&quot;:&quot;&lt;b64 enc. id of post&gt;&quot; }"/>
+    <hyperlink ref="C105" r:id="rId18" display="1. Open postman 2. Send a request to https://www.roysshack.hu/update_stock_admin with the body {  &quot;user_id&quot;:&quot;&lt;b64 enc. id of user&gt;&quot;, &quot;session_token&quot;:&quot;&lt;b64 enc. session token of user&gt;&quot;, &quot;post_id&quot;:&quot;&lt;b64 enc. id of post&gt;&quot; }, and no auth header"/>
+    <hyperlink ref="C106" r:id="rId19" display="1. Open postman 2. Send a request to https://www.roysshack.hu/update_stock_admin with the body {  &quot;user_id&quot;:&quot;&lt;b64 enc. id of user&gt;&quot;, &quot;session_token&quot;:&quot;&lt;b64 enc. session token of user&gt;&quot;, &quot;post_id&quot;:"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>